<commit_message>
Sprint 1: Next.js scaffold, database schema, policy and utilities
- Next.js 16 app with Tailwind; libSQL client (local file or Turso)
- Schema for source data, import bookkeeping, alerts, cases, decisions
- Triggers make alerts, cases and decisions immutable
- config/policy.json holds every detector weight and threshold
- Normalisation, hashing, robust statistics and union-find utilities
- 15 vitest tests (utilities + DB integrity)
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -572,7 +572,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>3bc9253</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
@@ -604,12 +608,20 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>15 tests pass; build OK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1035,11 +1047,15 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
     </row>
@@ -1066,13 +1082,21 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Raw SQL via @libsql/client instead of Drizzle</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1097,11 +1121,15 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
     </row>
@@ -1128,11 +1156,15 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
     </row>
@@ -1159,11 +1191,15 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
     </row>
@@ -2711,7 +2747,11 @@
         </is>
       </c>
       <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Triggers in place (tests/db.test.ts); end-to-end check after S4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F21"/>

</xml_diff>

<commit_message>
Sprint 2: seeded synthetic data generator and sample datasets
scripts/generate.ts builds linked customers, accounts, transactions,
logins and loan applications with planted fraud (S1-S6) and legitimate
lookalikes (L1-L4). Each seed writes CSV, XLSX and JSON, an error-demo
file, an alternate-header file and ground_truth.json (evaluation only).
Seeds 1-3 committed; output is deterministic per seed.
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -616,7 +616,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>f98e054</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>15 tests pass; build OK</t>
@@ -652,12 +656,20 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Seeds 1–3: 320 customers, ~4.5k txns, ~4k logins, 124 loans, 18 truth items each; deterministic</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1226,11 +1238,15 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
     </row>
@@ -1257,11 +1273,15 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
     </row>
@@ -1288,11 +1308,15 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
     </row>
@@ -1319,11 +1343,15 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
     </row>

</xml_diff>

<commit_message>
Sprint 3: ingestion pipeline and APIs
- CSV, multi-sheet XLSX and JSON (array or keyed object) parsing
- Header aliases and dataset-type detection with an optional override
- Per-field validation and normalisation; every row lands in exactly one
  bucket (accepted / rejected / duplicate) with warnings for orphans
- ID conflicts rejected, identical re-uploads counted as duplicates
- APIs: /api/ingest, /api/samples, /api/samples/load, /api/batches,
  /api/batches/[id]/errors (CSV issue report)
- 8 ingestion tests (23 total); smoke-tested against next start
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -664,7 +664,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>ddd79db</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Seeds 1–3: 320 customers, ~4.5k txns, ~4k logins, 124 loans, 18 truth items each; deterministic</t>
@@ -700,12 +704,20 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>23 tests pass; API smoke-tested on next start</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1378,11 +1390,15 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
     </row>
@@ -1409,11 +1425,15 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
     </row>
@@ -1440,13 +1460,21 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Explicit field validators (clear per-field messages); zod for API bodies</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1471,11 +1499,15 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
     </row>
@@ -1502,11 +1534,15 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
     </row>
@@ -2339,11 +2375,19 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>tests/ingest.test.ts</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2363,11 +2407,19 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>tests/ingest.test.ts</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2387,11 +2439,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>tests/ingest.test.ts</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2411,11 +2471,19 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>tests/ingest.test.ts</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sprint 4: detection engine, scoring, cross-system correlation and cases
- FD-01 suspicious transfer: robust baselines, new beneficiary, rapid
  succession, drain, login risk, mule fan-in; norm/tenure mitigations
- FD-02 shared device with household and long-standing-use mitigations
- FD-03 account takeover as an event sequence (burst, device, follow-on)
- FD-05 loan rings via union-find over shared identity attributes
- FD-06 cross-system correlation; cases group alerts sharing entities
- Score = signals - mitigations with severity floors; deterministic
  fingerprints make re-runs idempotent; alerts immutable
- Evaluator against ground_truth.json; /api/detect, /api/policy
- 39 tests: 11/11 fraud and 7/7 lookalikes on seeds 1-3
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -712,7 +712,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>eba6588</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>23 tests pass; API smoke-tested on next start</t>
@@ -748,12 +752,20 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>39 tests; 11/11 fraud, 7/7 lookalikes on 3 seeds; precision 79–92%; ~70 ms/run</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1569,11 +1581,15 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
     </row>
@@ -1600,11 +1616,15 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
     </row>
@@ -1631,11 +1651,15 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
     </row>
@@ -1662,11 +1686,15 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
     </row>
@@ -1693,11 +1721,15 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
     </row>
@@ -1724,11 +1756,15 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
     </row>
@@ -1755,11 +1791,15 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
     </row>
@@ -1786,13 +1826,21 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Cases group every Medium/High alert sharing an entity; FD-06 only when a group spans ≥2 customers or products</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1817,11 +1865,15 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
     </row>
@@ -2503,11 +2555,19 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>config/policy.json; Rules page in S6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2527,11 +2587,19 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2551,11 +2619,19 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2575,11 +2651,19 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2599,11 +2683,19 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2623,11 +2715,19 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2647,11 +2747,19 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2671,11 +2779,19 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2839,13 +2955,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Triggers in place (tests/db.test.ts); end-to-end check after S4</t>
+          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 5: dashboard, ingestion, alerts list and alert detail screens
- App shell with navigation; light/dark design tokens
- Dashboard: records processed, rejected rows, flagged events, open
  cases, risk distribution, categories and products, recent High alerts
- Ingest: bundled sample picker, multi-file upload with type override,
  per-dataset result cards (mapping, buckets, issues), import history
- Alerts: escalated / reviewed / all tabs and filters for customer,
  transaction, product, risk level, detector and date range
- Alert detail: score working, underlying event, why-flagged table,
  linked alerts, supporting records with source file and row
- APIs: /api/alerts, /api/alerts/[id], /api/dashboard
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -760,7 +760,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>b5d47e7</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>39 tests; 11/11 fraud, 7/7 lookalikes on 3 seeds; precision 79–92%; ~70 ms/run</t>
@@ -796,12 +800,20 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Screens checked in Playwright at 1440/390 px, light + dark; no overflow</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1900,11 +1912,15 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
     </row>
@@ -1931,13 +1947,21 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Charts as plain HTML bars (Recharts dropped): status colours + labels for risk, single hue for categories</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1962,11 +1986,15 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
     </row>
@@ -1993,11 +2021,15 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
     </row>
@@ -2024,11 +2056,15 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
@@ -2403,11 +2439,19 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ingest screen: sample picker + upload (screenshot-checked)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2811,11 +2855,19 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Why-flagged table with weights, details, evidence links</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2835,11 +2887,19 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard: records, flagged, risk distribution, categories, products</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2859,11 +2919,19 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>All 6 filters checked against /api/alerts on seed 3</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2883,11 +2951,19 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Alert detail: underlying event, reasons, source rows with file:row</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sprint 6: cases, decisions, customer investigation, rules and evaluation
- Case queue (open/closed/all) and case detail with classification,
  member alerts (read-only), connection reasons, merged timeline and
  supporting records
- Append-only decisions: Requires investigation, Escalate, False
  positive, Dismiss; optional risk/category reclassification; note
  required to close; original alerts never change
- Customer page: profile, devices with co-users, accounts, loans,
  alerts and a unified cross-system timeline
- Rules page rendered from config/policy.json
- Evaluation page scoring the latest run against a ground-truth file
- APIs: /api/cases, /api/cases/[id], /api/cases/[id]/decisions,
  /api/customers/[id], /api/evaluate; 45 tests
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -808,7 +808,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>ec2d613</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Screens checked in Playwright at 1440/390 px, light + dark; no overflow</t>
@@ -844,12 +848,20 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>45 tests; browser E2E: decision persists after reload; evaluation 11/11, 7/7 on seed 3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2091,11 +2103,15 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
@@ -2122,11 +2138,15 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
     </row>
@@ -2153,11 +2173,15 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
     </row>
@@ -2184,11 +2208,15 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
     </row>
@@ -2215,11 +2243,15 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
     </row>
@@ -2609,7 +2641,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>config/policy.json; Rules page in S6</t>
+          <t>config/policy.json rendered on /rules</t>
         </is>
       </c>
     </row>
@@ -2983,11 +3015,19 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Case: ID, customer/account, category, risk, evidence, status (tests/cases.test.ts)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3007,11 +3047,19 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Not verified</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Decision form; persisted across reload in browser E2E</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3041,7 +3089,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>tests/detect.test.ts + tests/integrity.test.ts (seeds 1–3)</t>
+          <t>Alerts byte-identical after decision + reclassification (tests/cases.test.ts)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 7: hardening, smoke test and documentation
- Reset workspace API and button (confirmation required)
- App-level error and not-found pages
- scripts/smoke.mjs: end-to-end API check of the demo flow (17 checks)
- README (run, data, architecture, API), KNOWN_LIMITATIONS, .env.example

Deployment is pending: it needs a hosted Turso database.
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -856,7 +856,11 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>a4f28f5</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t>45 tests; browser E2E: decision persists after reload; evaluation 11/11, 7/7 on seed 3</t>
@@ -892,12 +896,16 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Everything except deployment done</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2278,13 +2286,21 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Reset API + button; error/not-found pages; Next control-flow errors rethrown</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2309,11 +2325,15 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
     </row>
@@ -2340,13 +2360,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Needs go-ahead to publish + a Turso DB (Vercel CLI logged in as thanush-41; turso CLI not installed)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2371,13 +2395,21 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>scripts/smoke.mjs: 17/17 checks on seed 3 + browser E2E of decision flow</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I40"/>

</xml_diff>

<commit_message>
Add FD-04 identity detector and phishing-takeover detection
Closes two gaps against the problem statement:
- Scenario 1 (identity fraud, synthetic profiles): FD-04 links customers
  sharing a national ID, phone or email; scores ID reuse, clustered
  onboarding, unrelated identities and implausible attributes, with a
  household mitigation and an ID-reuse floor
- Scenario 3 (account takeover): FD-03 also starts from a successful
  login on a new device in a new location, so phished sessions with no
  failed logins (password reset -> new beneficiary -> transfer) are caught
- Generator: S7 synthetic identities, S8 phishing takeover, L5 household
  sharing a phone; seeds regenerated
- Seeds 1-3: 14/14 fraud, 8/8 lookalikes; 45 tests and 17 smoke checks pass
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -900,10 +900,14 @@
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>40c7b07</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Everything except deployment done</t>
+          <t>Post-review: FD-04 identity detector + FD-03 phishing anchor added (14/14, 8/8). Deploy pending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add insurance claims, FD-07 claim-fraud detector and richer data fields
Scenario 4 (cross-system with insurance) and better classification inputs:
- New insurance_claims dataset (ingest, aliases, validation, evidence,
  timelines, customer page); claims link into FD-02 and FD-06
- FD-07 scores duplicate documents/incidents, early claims, near sum
  insured, late reporting, claim frequency, shared payout accounts and
  provider clustering, with household and clean-history mitigations
- Richer fields: occupation and declared income on customers; stated
  income, employer and purpose on loans; FD-05 income-mismatch signal
- Generator: insurance policies and background claims; S9 claims paid
  into the loan ring's account, S10 double-dipping, L6 household payout
- Existing databases get the new columns via idempotent migrations
- Seeds 1-3: 17/17 fraud, 9/9 lookalikes; 45 tests, 17 smoke checks pass
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -902,12 +902,12 @@
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>40c7b07</t>
+          <t>145ed64</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Post-review: FD-04 identity detector + FD-03 phishing anchor added (14/14, 8/8). Deploy pending.</t>
+          <t>Added insurance claims (FD-07), richer fields, income mismatch; 17/17 fraud, 9/9 lookalikes. Deploy pending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Sprint 7 done (deployed, verified on production)
</commit_message>
<xml_diff>
--- a/SPRINTS.xlsx
+++ b/SPRINTS.xlsx
@@ -896,18 +896,22 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>145ed64</t>
+          <t>eb79df4</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Added insurance claims (FD-07), richer fields, income mismatch; 17/17 fraud, 9/9 lookalikes. Deploy pending.</t>
+          <t>Deployed; Reviews 1-2 addressed; 18/18 fraud, 10/10 lookalikes, 59 tests</t>
         </is>
       </c>
     </row>
@@ -2364,15 +2368,19 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Needs go-ahead to publish + a Turso DB (Vercel CLI logged in as thanush-41; turso CLI not installed)</t>
+          <t>Live: https://trace-x-rouge-rho.vercel.app (Vercel + Turso); smoke 20/20 and browser E2E pass on prod</t>
         </is>
       </c>
     </row>

</xml_diff>